<commit_message>
(Testing Documentation) verified board amplifies INPUT 1Hz (+-15mV) differential signal with 2.5V offset to ~=(0-3V) -(TODO)Noted attenuation of input signal as frequency increases
</commit_message>
<xml_diff>
--- a/Revision01/Testing/TestingResults.xlsx
+++ b/Revision01/Testing/TestingResults.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Parry\Documents\GitHub\BCIT-BAJA-DAQ\Revision01\Testing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Parry\Documents\GITHUB_desktop\BCIT-BAJA-DAQ\Revision01\Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A507D0C-605A-48E6-AA62-0CDAF2123C3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A440E053-D93C-45FA-A571-526CBE1E106B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{020E14A9-CA64-4B08-B51B-4D8FA57B006C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{020E14A9-CA64-4B08-B51B-4D8FA57B006C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Screenshot" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Testing procedure</t>
   </si>
@@ -66,6 +67,51 @@
   </si>
   <si>
     <t>Expected(V)</t>
+  </si>
+  <si>
+    <t>Measuring INA333 output</t>
+  </si>
+  <si>
+    <t>Input 0V differential</t>
+  </si>
+  <si>
+    <t>Attach strainGauge 0lbs of force</t>
+  </si>
+  <si>
+    <t>Get linear response for force applied</t>
+  </si>
+  <si>
+    <t>Test setup</t>
+  </si>
+  <si>
+    <t>INPUT</t>
+  </si>
+  <si>
+    <t>SCOPE MEASUREMENT OF INPUT</t>
+  </si>
+  <si>
+    <t>BOARD 1</t>
+  </si>
+  <si>
+    <t>1Hz</t>
+  </si>
+  <si>
+    <t>1HZ Sin wave MAX 15mV differential(2.5V offset)</t>
+  </si>
+  <si>
+    <t>1Hz Sin wave MIN Input - 15mV differential (2.5V offset)</t>
+  </si>
+  <si>
+    <t>100Hz</t>
+  </si>
+  <si>
+    <t>10Hz</t>
+  </si>
+  <si>
+    <t>1K Hz</t>
+  </si>
+  <si>
+    <t>1KHZ input wave measured</t>
   </si>
 </sst>
 </file>
@@ -124,15 +170,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -159,6 +204,319 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>14311</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>9524</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>180974</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>180213</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0603828-51F5-68E7-E5D3-F12CE114501E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6719911" y="390524"/>
+          <a:ext cx="6872263" cy="4171189"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>47626</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>57149</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>58113</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{37EA401F-394C-3AC7-9FAB-448061F6621E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="47626" y="438149"/>
+          <a:ext cx="6696074" cy="4191964"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>196766</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>255207</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>96028</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A34C02AB-689E-ACBE-8D31-16635CCCF969}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="196766" y="5862888"/>
+          <a:ext cx="9182388" cy="5863666"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>320721</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>59430</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>60</xdr:col>
+      <xdr:colOff>491085</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>169081</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{40A9CBFC-D057-9796-6ABF-717EFB581A20}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="27782558" y="5717050"/>
+          <a:ext cx="9293708" cy="5767272"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>115692</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>81523</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>298374</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>82515</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8C094799-0C6C-BB26-37A6-75A31C0FAB56}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18454186" y="5739143"/>
+          <a:ext cx="9306025" cy="5658613"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>100264</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>75197</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>112083</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>91807</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1A4B67C-F36A-4549-808A-774446F3CEAC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9315415" y="5732817"/>
+          <a:ext cx="9135162" cy="5674231"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>46</xdr:col>
+      <xdr:colOff>42694</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>63501</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>239763</xdr:colOff>
+      <xdr:row>98</xdr:row>
+      <xdr:rowOff>66545</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A315CF00-70A0-9481-1E82-8B7BDD9ADCF1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="28173194" y="12636501"/>
+          <a:ext cx="9341069" cy="6099044"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -478,57 +836,57 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{743264EB-18C6-49E4-B5B2-50CC06CB0E0E}">
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.5703125" customWidth="1"/>
+    <col min="1" max="1" width="49.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" t="s">
         <v>5</v>
       </c>
       <c r="B3">
@@ -539,7 +897,7 @@
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4">
@@ -585,13 +943,61 @@
       </c>
       <c r="C10">
         <v>1.67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13">
+        <v>1.67</v>
+      </c>
+      <c r="C13">
+        <v>1.67</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14">
+        <v>3.1</v>
+      </c>
+      <c r="C14">
+        <v>3.1909999999999998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15">
+        <v>0.1</v>
+      </c>
+      <c r="C15">
+        <v>0.1578</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
-  <conditionalFormatting sqref="C3:C10">
+  <conditionalFormatting sqref="C3:C19">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>$B$3</formula>
     </cfRule>
@@ -599,4 +1005,56 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21B1AB74-EBC0-4F0D-8BBC-5FC355088006}">
+  <dimension ref="A1:AU66"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="L2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>22</v>
+      </c>
+      <c r="AF29" t="s">
+        <v>21</v>
+      </c>
+      <c r="AR29" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="66" spans="47:47" x14ac:dyDescent="0.25">
+      <c r="AU66" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
was able to verify second board works up to 1KHz, however test results are very inconsistent.
</commit_message>
<xml_diff>
--- a/Revision01/Testing/TestingResults.xlsx
+++ b/Revision01/Testing/TestingResults.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Parry\Documents\GITHUB_desktop\BCIT-BAJA-DAQ\Revision01\Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A440E053-D93C-45FA-A571-526CBE1E106B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4398A4B3-102D-4FE6-9C12-46511DF66B86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{020E14A9-CA64-4B08-B51B-4D8FA57B006C}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
   <si>
     <t>Testing procedure</t>
   </si>
@@ -112,6 +112,27 @@
   </si>
   <si>
     <t>1KHZ input wave measured</t>
+  </si>
+  <si>
+    <t>BOARD 2</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>BOARD 1 ATTEMPT 2</t>
+  </si>
+  <si>
+    <t>10hZ</t>
+  </si>
+  <si>
+    <t>1Khz</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">??????????????? Wtf tested twice…. </t>
   </si>
 </sst>
 </file>
@@ -474,16 +495,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>46</xdr:col>
-      <xdr:colOff>42694</xdr:colOff>
-      <xdr:row>66</xdr:row>
-      <xdr:rowOff>63501</xdr:rowOff>
+      <xdr:col>62</xdr:col>
+      <xdr:colOff>317861</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>127001</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>61</xdr:col>
-      <xdr:colOff>239763</xdr:colOff>
-      <xdr:row>98</xdr:row>
-      <xdr:rowOff>66545</xdr:rowOff>
+      <xdr:col>77</xdr:col>
+      <xdr:colOff>514930</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>130045</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -506,8 +527,360 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28173194" y="12636501"/>
-          <a:ext cx="9341069" cy="6099044"/>
+          <a:off x="38460194" y="5080001"/>
+          <a:ext cx="9404569" cy="6099044"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>94881</xdr:colOff>
+      <xdr:row>90</xdr:row>
+      <xdr:rowOff>179457</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FDF2AB1D-33F3-0648-F3E7-FB899230355F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="11982174"/>
+          <a:ext cx="9288577" cy="5590761"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>400924</xdr:colOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>78971</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>46</xdr:col>
+      <xdr:colOff>538099</xdr:colOff>
+      <xdr:row>82</xdr:row>
+      <xdr:rowOff>181918</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A7D7FB6B-F92A-F00B-1352-82E4DA267A08}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19178781" y="12131012"/>
+          <a:ext cx="9176206" cy="3990702"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>136073</xdr:colOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>58316</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>354191</xdr:colOff>
+      <xdr:row>90</xdr:row>
+      <xdr:rowOff>140730</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Picture 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ADA57B06-2516-34F1-587A-0DB8BD1A28E4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9272297" y="12110357"/>
+          <a:ext cx="9859751" cy="5525271"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>388775</xdr:colOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>77755</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>578315</xdr:colOff>
+      <xdr:row>90</xdr:row>
+      <xdr:rowOff>150643</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Picture 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0CD7278E-B7FB-9C89-CA7E-1F7870D0719D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="27603061" y="12129796"/>
+          <a:ext cx="9831172" cy="5515745"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>95</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>31721</xdr:colOff>
+      <xdr:row>125</xdr:row>
+      <xdr:rowOff>51784</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Picture 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9D64FDFE-ABA7-8EF9-D8A9-104E73D9F8E7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="17513710"/>
+          <a:ext cx="9326277" cy="5582429"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>95</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>213324</xdr:colOff>
+      <xdr:row>125</xdr:row>
+      <xdr:rowOff>51784</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Picture 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C211FF7E-FFDF-939C-8B72-208E21D9B219}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9294556" y="17513710"/>
+          <a:ext cx="9431066" cy="5582429"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>95</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>46</xdr:col>
+      <xdr:colOff>108536</xdr:colOff>
+      <xdr:row>125</xdr:row>
+      <xdr:rowOff>23205</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Picture 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CEE9EE85-A535-61D8-E001-5D84DCC2339A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19126815" y="17513710"/>
+          <a:ext cx="9326277" cy="5553850"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>46</xdr:col>
+      <xdr:colOff>199718</xdr:colOff>
+      <xdr:row>94</xdr:row>
+      <xdr:rowOff>138266</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>298726</xdr:colOff>
+      <xdr:row>124</xdr:row>
+      <xdr:rowOff>170997</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="Picture 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D8A64B57-B9A9-95A8-2D74-BCC98EE9F001}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="28544274" y="17467621"/>
+          <a:ext cx="9316750" cy="5563376"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1009,7 +1382,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21B1AB74-EBC0-4F0D-8BBC-5FC355088006}">
-  <dimension ref="A1:AU66"/>
+  <dimension ref="A1:BL95"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1028,12 +1401,17 @@
         <v>16</v>
       </c>
     </row>
-    <row r="27" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:64" x14ac:dyDescent="0.25">
+      <c r="BL26" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="29" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>18</v>
       </c>
@@ -1047,9 +1425,46 @@
         <v>23</v>
       </c>
     </row>
-    <row r="66" spans="47:47" x14ac:dyDescent="0.25">
-      <c r="AU66" t="s">
-        <v>24</v>
+    <row r="60" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AX60" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="61" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="A61" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="62" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="63" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AE63" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="94" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>27</v>
+      </c>
+      <c r="F94" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF94" t="s">
+        <v>21</v>
+      </c>
+      <c r="AU94" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="95" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="P95" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q95" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
(hardware Testing) board 1 and 2 have been verified to work: bug is attributed to testing software bug.
- the bug found was toggling input W1 and W2 on and off with same settings at like 1 Khz results in varying amplitudes, even though the
settings remain at +-10mV
</commit_message>
<xml_diff>
--- a/Revision01/Testing/TestingResults.xlsx
+++ b/Revision01/Testing/TestingResults.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Parry\Documents\GITHUB_desktop\BCIT-BAJA-DAQ\Revision01\Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4398A4B3-102D-4FE6-9C12-46511DF66B86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4352C716-D818-4752-BC54-B7F922C8D0FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{020E14A9-CA64-4B08-B51B-4D8FA57B006C}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
   <si>
     <t>Testing procedure</t>
   </si>
@@ -111,28 +111,10 @@
     <t>1K Hz</t>
   </si>
   <si>
-    <t>1KHZ input wave measured</t>
-  </si>
-  <si>
     <t>BOARD 2</t>
   </si>
   <si>
     <t>x</t>
-  </si>
-  <si>
-    <t>BOARD 1 ATTEMPT 2</t>
-  </si>
-  <si>
-    <t>10hZ</t>
-  </si>
-  <si>
-    <t>1Khz</t>
-  </si>
-  <si>
-    <t>s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">??????????????? Wtf tested twice…. </t>
   </si>
 </sst>
 </file>
@@ -231,6 +213,55 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>335139</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>19109</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>36125</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>114193</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9B7AF9D7-BB8D-05D3-FE10-649F243170D5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9566158" y="207257"/>
+          <a:ext cx="9484689" cy="6492121"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>14311</xdr:colOff>
       <xdr:row>2</xdr:row>
@@ -238,9 +269,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>180974</xdr:colOff>
+      <xdr:colOff>5824</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>180213</xdr:rowOff>
+      <xdr:rowOff>129588</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -407,50 +438,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>115692</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>81523</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>45</xdr:col>
-      <xdr:colOff>298374</xdr:colOff>
-      <xdr:row>58</xdr:row>
-      <xdr:rowOff>82515</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Picture 7">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8C094799-0C6C-BB26-37A6-75A31C0FAB56}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="18454186" y="5739143"/>
-          <a:ext cx="9306025" cy="5658613"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>15</xdr:col>
       <xdr:colOff>100264</xdr:colOff>
       <xdr:row>29</xdr:row>
@@ -495,23 +482,67 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>62</xdr:col>
-      <xdr:colOff>317861</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>127001</xdr:rowOff>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>448236</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>56029</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>77</xdr:col>
-      <xdr:colOff>514930</xdr:colOff>
-      <xdr:row>58</xdr:row>
-      <xdr:rowOff>130045</xdr:rowOff>
+      <xdr:col>46</xdr:col>
+      <xdr:colOff>7486</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>6455</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Picture 9">
+        <xdr:cNvPr id="5" name="Picture 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A315CF00-70A0-9481-1E82-8B7BDD9ADCF1}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{911B45B2-11C0-BD7E-DFB5-435504CB5975}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19021986" y="5939117"/>
+          <a:ext cx="9420426" cy="5629126"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>196103</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>84044</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>186545</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>11920</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="29" name="Picture 28">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A6E7E4A0-3EDD-4D81-8763-10D26B8BF47B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -527,8 +558,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="38460194" y="5080001"/>
-          <a:ext cx="9404569" cy="6099044"/>
+          <a:off x="196103" y="12438529"/>
+          <a:ext cx="9319339" cy="5614862"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -539,23 +570,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>62</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>585467</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>84044</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>94881</xdr:colOff>
-      <xdr:row>90</xdr:row>
-      <xdr:rowOff>179457</xdr:rowOff>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>53156</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>59552</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
+        <xdr:cNvPr id="30" name="Picture 29">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FDF2AB1D-33F3-0648-F3E7-FB899230355F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E5EE00AC-B505-4F98-AFCC-EE46BA17410F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -571,8 +602,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="11982174"/>
-          <a:ext cx="9288577" cy="5590761"/>
+          <a:off x="9914364" y="12438529"/>
+          <a:ext cx="9328866" cy="5662494"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -583,23 +614,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>31</xdr:col>
-      <xdr:colOff>400924</xdr:colOff>
-      <xdr:row>62</xdr:row>
-      <xdr:rowOff>78971</xdr:rowOff>
+      <xdr:col>46</xdr:col>
+      <xdr:colOff>397949</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>47850</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>46</xdr:col>
-      <xdr:colOff>538099</xdr:colOff>
-      <xdr:row>82</xdr:row>
-      <xdr:rowOff>181918</xdr:rowOff>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>296178</xdr:colOff>
+      <xdr:row>91</xdr:row>
+      <xdr:rowOff>108668</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="Picture 10">
+        <xdr:cNvPr id="31" name="Picture 30">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A7D7FB6B-F92A-F00B-1352-82E4DA267A08}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3BFFFDDB-E957-496F-9E34-A8B8693556C4}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -615,8 +646,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="19178781" y="12131012"/>
-          <a:ext cx="9176206" cy="3990702"/>
+          <a:off x="28832875" y="12402335"/>
+          <a:ext cx="9143082" cy="5551701"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -627,23 +658,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>136073</xdr:colOff>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>190418</xdr:colOff>
       <xdr:row>62</xdr:row>
-      <xdr:rowOff>58316</xdr:rowOff>
+      <xdr:rowOff>189200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>31</xdr:col>
-      <xdr:colOff>354191</xdr:colOff>
-      <xdr:row>90</xdr:row>
-      <xdr:rowOff>140730</xdr:rowOff>
+      <xdr:col>46</xdr:col>
+      <xdr:colOff>271615</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>71402</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="Picture 11">
+        <xdr:cNvPr id="32" name="Picture 31">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ADA57B06-2516-34F1-587A-0DB8BD1A28E4}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0D757854-3493-4103-9AA4-1B68B8D7E09F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -659,228 +690,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9272297" y="12110357"/>
-          <a:ext cx="9859751" cy="5525271"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>45</xdr:col>
-      <xdr:colOff>388775</xdr:colOff>
-      <xdr:row>62</xdr:row>
-      <xdr:rowOff>77755</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>61</xdr:col>
-      <xdr:colOff>578315</xdr:colOff>
-      <xdr:row>90</xdr:row>
-      <xdr:rowOff>150643</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="13" name="Picture 12">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0CD7278E-B7FB-9C89-CA7E-1F7870D0719D}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="27603061" y="12129796"/>
-          <a:ext cx="9831172" cy="5515745"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>95</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>31721</xdr:colOff>
-      <xdr:row>125</xdr:row>
-      <xdr:rowOff>51784</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="14" name="Picture 13">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9D64FDFE-ABA7-8EF9-D8A9-104E73D9F8E7}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="17513710"/>
-          <a:ext cx="9326277" cy="5582429"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>95</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>213324</xdr:colOff>
-      <xdr:row>125</xdr:row>
-      <xdr:rowOff>51784</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="16" name="Picture 15">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C211FF7E-FFDF-939C-8B72-208E21D9B219}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9294556" y="17513710"/>
-          <a:ext cx="9431066" cy="5582429"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>31</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>95</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>46</xdr:col>
-      <xdr:colOff>108536</xdr:colOff>
-      <xdr:row>125</xdr:row>
-      <xdr:rowOff>23205</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="17" name="Picture 16">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CEE9EE85-A535-61D8-E001-5D84DCC2339A}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="19126815" y="17513710"/>
-          <a:ext cx="9326277" cy="5553850"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>46</xdr:col>
-      <xdr:colOff>199718</xdr:colOff>
-      <xdr:row>94</xdr:row>
-      <xdr:rowOff>138266</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>61</xdr:col>
-      <xdr:colOff>298726</xdr:colOff>
-      <xdr:row>124</xdr:row>
-      <xdr:rowOff>170997</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="18" name="Picture 17">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D8A64B57-B9A9-95A8-2D74-BCC98EE9F001}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="28544274" y="17467621"/>
-          <a:ext cx="9316750" cy="5563376"/>
+          <a:off x="19380492" y="12347582"/>
+          <a:ext cx="9326049" cy="5765291"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1377,12 +1188,13 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21B1AB74-EBC0-4F0D-8BBC-5FC355088006}">
-  <dimension ref="A1:BL95"/>
+  <dimension ref="A1:AX63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1401,17 +1213,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:64" x14ac:dyDescent="0.25">
-      <c r="BL26" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="27" spans="1:64" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="29" spans="1:64" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>18</v>
       </c>
@@ -1427,12 +1234,12 @@
     </row>
     <row r="60" spans="1:50" x14ac:dyDescent="0.25">
       <c r="AX60" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="61" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="62" spans="1:50" x14ac:dyDescent="0.25">
@@ -1443,28 +1250,6 @@
     <row r="63" spans="1:50" x14ac:dyDescent="0.25">
       <c r="AE63" t="s">
         <v>21</v>
-      </c>
-    </row>
-    <row r="94" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>27</v>
-      </c>
-      <c r="F94" t="s">
-        <v>30</v>
-      </c>
-      <c r="AF94" t="s">
-        <v>21</v>
-      </c>
-      <c r="AU94" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="95" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="P95" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q95" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
(hardware Testing) attached strain gauge onto board 1 for basic testing
- offset voltage is about 1.44V rather than 1.67V
- bent strain gauge and saw change in voltage
</commit_message>
<xml_diff>
--- a/Revision01/Testing/TestingResults.xlsx
+++ b/Revision01/Testing/TestingResults.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Parry\Documents\GITHUB_desktop\BCIT-BAJA-DAQ\Revision01\Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4352C716-D818-4752-BC54-B7F922C8D0FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{379C5414-CBCC-4772-9BA6-D742E293BBC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{020E14A9-CA64-4B08-B51B-4D8FA57B006C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{020E14A9-CA64-4B08-B51B-4D8FA57B006C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
   <si>
     <t>Testing procedure</t>
   </si>
@@ -115,6 +115,15 @@
   </si>
   <si>
     <t>x</t>
+  </si>
+  <si>
+    <t>Attach real strain gauge test</t>
+  </si>
+  <si>
+    <t>offset voltage(V)</t>
+  </si>
+  <si>
+    <t>output voltage(V)</t>
   </si>
 </sst>
 </file>
@@ -1020,7 +1029,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{743264EB-18C6-49E4-B5B2-50CC06CB0E0E}">
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49.7109375" bestFit="1" customWidth="1"/>
@@ -1167,13 +1176,40 @@
         <v>0.1578</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18">
+        <v>1.67</v>
+      </c>
+      <c r="C18">
+        <v>1.444</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19">
+        <v>1.67</v>
+      </c>
+      <c r="C19">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1181,7 +1217,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
-  <conditionalFormatting sqref="C3:C19">
+  <conditionalFormatting sqref="C3:C21">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>$B$3</formula>
     </cfRule>

</xml_diff>